<commit_message>
#4494-PurchaseInvoice Module: pabi_account_report (Restart & Update Module) เพิ่มเงื่อนไขการออกรายงน https://mobileapp.nstda.or.th/redmine/issues/4494
</commit_message>
<xml_diff>
--- a/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
+++ b/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>PO Number</t>
   </si>
@@ -221,10 +221,13 @@
     <t>Invoice Status</t>
   </si>
   <si>
-    <t>Period</t>
-  </si>
-  <si>
     <t>Filter</t>
+  </si>
+  <si>
+    <t>Period Invoice</t>
+  </si>
+  <si>
+    <t>Period PO</t>
   </si>
 </sst>
 </file>
@@ -599,7 +602,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:BL11"/>
+  <dimension ref="A1:BM11"/>
   <sheetFormatPr defaultColWidth="14.125" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -624,30 +627,30 @@
     <col min="28" max="28" width="13.875" customWidth="1"/>
     <col min="29" max="29" width="12.5" style="1" customWidth="1"/>
     <col min="30" max="30" width="42.375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="16.25" customWidth="1"/>
-    <col min="32" max="33" width="16.25" style="1" customWidth="1"/>
-    <col min="34" max="41" width="16.25" customWidth="1"/>
-    <col min="42" max="43" width="19.5" customWidth="1"/>
-    <col min="44" max="45" width="16.25" customWidth="1"/>
-    <col min="46" max="46" width="16.625" customWidth="1"/>
-    <col min="47" max="47" width="17.875" customWidth="1"/>
-    <col min="48" max="54" width="16.25" customWidth="1"/>
-    <col min="55" max="55" width="21.875" customWidth="1"/>
-    <col min="56" max="56" width="17.875" customWidth="1"/>
-    <col min="57" max="58" width="16.25" customWidth="1"/>
-    <col min="59" max="59" width="9.875" customWidth="1"/>
-    <col min="60" max="60" width="23" customWidth="1"/>
-    <col min="61" max="61" width="10.25" customWidth="1"/>
-    <col min="62" max="62" width="16.25" customWidth="1"/>
-    <col min="63" max="63" width="9.75" customWidth="1"/>
+    <col min="31" max="32" width="16.25" customWidth="1"/>
+    <col min="33" max="34" width="16.25" style="1" customWidth="1"/>
+    <col min="35" max="42" width="16.25" customWidth="1"/>
+    <col min="43" max="44" width="19.5" customWidth="1"/>
+    <col min="45" max="46" width="16.25" customWidth="1"/>
+    <col min="47" max="47" width="16.625" customWidth="1"/>
+    <col min="48" max="48" width="17.875" customWidth="1"/>
+    <col min="49" max="55" width="16.25" customWidth="1"/>
+    <col min="56" max="56" width="21.875" customWidth="1"/>
+    <col min="57" max="57" width="17.875" customWidth="1"/>
+    <col min="58" max="59" width="16.25" customWidth="1"/>
+    <col min="60" max="60" width="9.875" customWidth="1"/>
+    <col min="61" max="61" width="23" customWidth="1"/>
+    <col min="62" max="62" width="10.25" customWidth="1"/>
+    <col min="63" max="63" width="16.25" customWidth="1"/>
+    <col min="64" max="64" width="9.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>45</v>
       </c>
@@ -658,8 +661,9 @@
       <c r="AC2"/>
       <c r="AD2"/>
       <c r="AE2" s="1"/>
-    </row>
-    <row r="3" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF2" s="1"/>
+    </row>
+    <row r="3" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
@@ -672,8 +676,9 @@
       <c r="AC3"/>
       <c r="AD3"/>
       <c r="AE3" s="1"/>
-    </row>
-    <row r="4" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF3" s="1"/>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
@@ -686,8 +691,9 @@
       <c r="AC4"/>
       <c r="AD4"/>
       <c r="AE4" s="1"/>
-    </row>
-    <row r="5" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF4" s="1"/>
+    </row>
+    <row r="5" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -700,8 +706,9 @@
       <c r="AC5"/>
       <c r="AD5"/>
       <c r="AE5" s="1"/>
-    </row>
-    <row r="6" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF5" s="1"/>
+    </row>
+    <row r="6" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
@@ -714,8 +721,9 @@
       <c r="AC6"/>
       <c r="AD6"/>
       <c r="AE6" s="1"/>
-    </row>
-    <row r="7" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF6" s="1"/>
+    </row>
+    <row r="7" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
@@ -726,8 +734,9 @@
       <c r="AC7"/>
       <c r="AD7"/>
       <c r="AE7" s="1"/>
-    </row>
-    <row r="8" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF7" s="1"/>
+    </row>
+    <row r="8" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
@@ -738,10 +747,11 @@
       <c r="AC8"/>
       <c r="AD8"/>
       <c r="AE8" s="1"/>
-    </row>
-    <row r="9" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF8" s="1"/>
+    </row>
+    <row r="9" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
@@ -750,8 +760,9 @@
       <c r="AC9"/>
       <c r="AD9"/>
       <c r="AE9" s="1"/>
-    </row>
-    <row r="10" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF9" s="1"/>
+    </row>
+    <row r="10" spans="1:65" x14ac:dyDescent="0.2">
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
       <c r="AA10" s="1"/>
@@ -759,8 +770,9 @@
       <c r="AC10"/>
       <c r="AD10"/>
       <c r="AE10" s="1"/>
-    </row>
-    <row r="11" spans="1:64" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="AF10" s="1"/>
+    </row>
+    <row r="11" spans="1:65" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>17</v>
       </c>
@@ -854,103 +866,106 @@
       <c r="AE11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AF11" s="8" t="s">
+      <c r="AF11" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="AG11" s="8" t="s">
+      <c r="AH11" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="AH11" s="8" t="s">
+      <c r="AI11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="AI11" s="5" t="s">
+      <c r="AJ11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="AJ11" s="8" t="s">
+      <c r="AK11" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="AK11" s="8" t="s">
+      <c r="AL11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AL11" s="5" t="s">
+      <c r="AM11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="AM11" s="8" t="s">
+      <c r="AN11" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="AN11" s="5" t="s">
+      <c r="AO11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AO11" s="5" t="s">
+      <c r="AP11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AP11" s="5" t="s">
+      <c r="AQ11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="AQ11" s="5" t="s">
+      <c r="AR11" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AR11" s="5" t="s">
+      <c r="AS11" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AS11" s="5" t="s">
+      <c r="AT11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="AT11" s="5" t="s">
+      <c r="AU11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AU11" s="5" t="s">
+      <c r="AV11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="AV11" s="5" t="s">
+      <c r="AW11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AW11" s="5" t="s">
+      <c r="AX11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="AX11" s="5" t="s">
+      <c r="AY11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AY11" s="5" t="s">
+      <c r="AZ11" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="AZ11" s="5" t="s">
+      <c r="BA11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="BA11" s="5" t="s">
+      <c r="BB11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="BB11" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="BC11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BD11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="BD11" s="5" t="s">
+      <c r="BE11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="BE11" s="5" t="s">
+      <c r="BF11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="BF11" s="5" t="s">
+      <c r="BG11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="BG11" s="5" t="s">
+      <c r="BH11" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="BH11" s="5" t="s">
+      <c r="BI11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="BI11" s="5" t="s">
+      <c r="BJ11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="BJ11" s="5" t="s">
+      <c r="BK11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="BK11" s="5" t="s">
+      <c r="BL11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="BL11" s="5" t="s">
+      <c r="BM11" s="5" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
#4494-PurchaseInvoice Module: pabi_account_report (Restart & Update Module) เพิ่มเงื่อนไขการออกรายงาน https://github.com/pabi2/pb2_addons/pull/1903
</commit_message>
<xml_diff>
--- a/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
+++ b/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
   <si>
     <t>PO Number</t>
   </si>
@@ -221,10 +221,13 @@
     <t>Invoice Status</t>
   </si>
   <si>
-    <t>Period</t>
-  </si>
-  <si>
     <t>Filter</t>
+  </si>
+  <si>
+    <t>Period Invoice</t>
+  </si>
+  <si>
+    <t>Period PO</t>
   </si>
 </sst>
 </file>
@@ -599,7 +602,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:BL11"/>
+  <dimension ref="A1:BM11"/>
   <sheetFormatPr defaultColWidth="14.125" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -624,30 +627,30 @@
     <col min="28" max="28" width="13.875" customWidth="1"/>
     <col min="29" max="29" width="12.5" style="1" customWidth="1"/>
     <col min="30" max="30" width="42.375" style="1" customWidth="1"/>
-    <col min="31" max="31" width="16.25" customWidth="1"/>
-    <col min="32" max="33" width="16.25" style="1" customWidth="1"/>
-    <col min="34" max="41" width="16.25" customWidth="1"/>
-    <col min="42" max="43" width="19.5" customWidth="1"/>
-    <col min="44" max="45" width="16.25" customWidth="1"/>
-    <col min="46" max="46" width="16.625" customWidth="1"/>
-    <col min="47" max="47" width="17.875" customWidth="1"/>
-    <col min="48" max="54" width="16.25" customWidth="1"/>
-    <col min="55" max="55" width="21.875" customWidth="1"/>
-    <col min="56" max="56" width="17.875" customWidth="1"/>
-    <col min="57" max="58" width="16.25" customWidth="1"/>
-    <col min="59" max="59" width="9.875" customWidth="1"/>
-    <col min="60" max="60" width="23" customWidth="1"/>
-    <col min="61" max="61" width="10.25" customWidth="1"/>
-    <col min="62" max="62" width="16.25" customWidth="1"/>
-    <col min="63" max="63" width="9.75" customWidth="1"/>
+    <col min="31" max="32" width="16.25" customWidth="1"/>
+    <col min="33" max="34" width="16.25" style="1" customWidth="1"/>
+    <col min="35" max="42" width="16.25" customWidth="1"/>
+    <col min="43" max="44" width="19.5" customWidth="1"/>
+    <col min="45" max="46" width="16.25" customWidth="1"/>
+    <col min="47" max="47" width="16.625" customWidth="1"/>
+    <col min="48" max="48" width="17.875" customWidth="1"/>
+    <col min="49" max="55" width="16.25" customWidth="1"/>
+    <col min="56" max="56" width="21.875" customWidth="1"/>
+    <col min="57" max="57" width="17.875" customWidth="1"/>
+    <col min="58" max="59" width="16.25" customWidth="1"/>
+    <col min="60" max="60" width="9.875" customWidth="1"/>
+    <col min="61" max="61" width="23" customWidth="1"/>
+    <col min="62" max="62" width="10.25" customWidth="1"/>
+    <col min="63" max="63" width="16.25" customWidth="1"/>
+    <col min="64" max="64" width="9.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:64" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:64" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>45</v>
       </c>
@@ -658,8 +661,9 @@
       <c r="AC2"/>
       <c r="AD2"/>
       <c r="AE2" s="1"/>
-    </row>
-    <row r="3" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF2" s="1"/>
+    </row>
+    <row r="3" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>11</v>
       </c>
@@ -672,8 +676,9 @@
       <c r="AC3"/>
       <c r="AD3"/>
       <c r="AE3" s="1"/>
-    </row>
-    <row r="4" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF3" s="1"/>
+    </row>
+    <row r="4" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>0</v>
       </c>
@@ -686,8 +691,9 @@
       <c r="AC4"/>
       <c r="AD4"/>
       <c r="AE4" s="1"/>
-    </row>
-    <row r="5" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF4" s="1"/>
+    </row>
+    <row r="5" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -700,8 +706,9 @@
       <c r="AC5"/>
       <c r="AD5"/>
       <c r="AE5" s="1"/>
-    </row>
-    <row r="6" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF5" s="1"/>
+    </row>
+    <row r="6" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>37</v>
       </c>
@@ -714,8 +721,9 @@
       <c r="AC6"/>
       <c r="AD6"/>
       <c r="AE6" s="1"/>
-    </row>
-    <row r="7" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF6" s="1"/>
+    </row>
+    <row r="7" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>47</v>
       </c>
@@ -726,8 +734,9 @@
       <c r="AC7"/>
       <c r="AD7"/>
       <c r="AE7" s="1"/>
-    </row>
-    <row r="8" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF7" s="1"/>
+    </row>
+    <row r="8" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>3</v>
       </c>
@@ -738,10 +747,11 @@
       <c r="AC8"/>
       <c r="AD8"/>
       <c r="AE8" s="1"/>
-    </row>
-    <row r="9" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF8" s="1"/>
+    </row>
+    <row r="9" spans="1:65" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
@@ -750,8 +760,9 @@
       <c r="AC9"/>
       <c r="AD9"/>
       <c r="AE9" s="1"/>
-    </row>
-    <row r="10" spans="1:64" x14ac:dyDescent="0.2">
+      <c r="AF9" s="1"/>
+    </row>
+    <row r="10" spans="1:65" x14ac:dyDescent="0.2">
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
       <c r="AA10" s="1"/>
@@ -759,8 +770,9 @@
       <c r="AC10"/>
       <c r="AD10"/>
       <c r="AE10" s="1"/>
-    </row>
-    <row r="11" spans="1:64" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="AF10" s="1"/>
+    </row>
+    <row r="11" spans="1:65" s="5" customFormat="1" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>17</v>
       </c>
@@ -854,103 +866,106 @@
       <c r="AE11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="AF11" s="8" t="s">
+      <c r="AF11" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="AG11" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="AG11" s="8" t="s">
+      <c r="AH11" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="AH11" s="8" t="s">
+      <c r="AI11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="AI11" s="5" t="s">
+      <c r="AJ11" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="AJ11" s="8" t="s">
+      <c r="AK11" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="AK11" s="8" t="s">
+      <c r="AL11" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="AL11" s="5" t="s">
+      <c r="AM11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="AM11" s="8" t="s">
+      <c r="AN11" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="AN11" s="5" t="s">
+      <c r="AO11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="AO11" s="5" t="s">
+      <c r="AP11" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="AP11" s="5" t="s">
+      <c r="AQ11" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="AQ11" s="5" t="s">
+      <c r="AR11" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="AR11" s="5" t="s">
+      <c r="AS11" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="AS11" s="5" t="s">
+      <c r="AT11" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="AT11" s="5" t="s">
+      <c r="AU11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="AU11" s="5" t="s">
+      <c r="AV11" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="AV11" s="5" t="s">
+      <c r="AW11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="AW11" s="5" t="s">
+      <c r="AX11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="AX11" s="5" t="s">
+      <c r="AY11" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="AY11" s="5" t="s">
+      <c r="AZ11" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="AZ11" s="5" t="s">
+      <c r="BA11" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="BA11" s="5" t="s">
+      <c r="BB11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="BB11" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="BC11" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="BD11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="BD11" s="5" t="s">
+      <c r="BE11" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="BE11" s="5" t="s">
+      <c r="BF11" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="BF11" s="5" t="s">
+      <c r="BG11" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="BG11" s="5" t="s">
+      <c r="BH11" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="BH11" s="5" t="s">
+      <c r="BI11" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="BI11" s="5" t="s">
+      <c r="BJ11" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="BJ11" s="5" t="s">
+      <c r="BK11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="BK11" s="5" t="s">
+      <c r="BL11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="BL11" s="5" t="s">
+      <c r="BM11" s="5" t="s">
         <v>59</v>
       </c>
     </row>

</xml_diff>

<commit_message>
#4494-PurchaseInvoice Module: pabi_account_report (Restart & Update Module) เพิ่มเงื่อนไขการออกรายงาน https://mobileapp.nstda.or.th/redmine/issues/4494
</commit_message>
<xml_diff>
--- a/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
+++ b/pabi_account_report/xlsx_template/xlsx_report_purchase_invoice_plan.xlsx
@@ -227,15 +227,16 @@
     <t>Period Invoice</t>
   </si>
   <si>
-    <t>Period PO</t>
+    <t>Period KV</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="187" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="188" formatCode="0.00000"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -297,7 +298,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -315,6 +316,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="188" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="188" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -605,22 +610,23 @@
   <dimension ref="A1:BM11"/>
   <sheetFormatPr defaultColWidth="14.125" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10" customWidth="1"/>
-    <col min="2" max="2" width="12.875" customWidth="1"/>
-    <col min="3" max="3" width="16.25" customWidth="1"/>
-    <col min="4" max="4" width="16.25" style="3" customWidth="1"/>
-    <col min="5" max="5" width="8.875" customWidth="1"/>
+    <col min="1" max="1" width="8.375" customWidth="1"/>
+    <col min="2" max="2" width="13.125" customWidth="1"/>
+    <col min="3" max="3" width="15.25" customWidth="1"/>
+    <col min="4" max="4" width="15.25" style="3" customWidth="1"/>
+    <col min="5" max="5" width="7.5" customWidth="1"/>
     <col min="6" max="7" width="16.25" customWidth="1"/>
     <col min="8" max="8" width="21.5" customWidth="1"/>
     <col min="9" max="9" width="16.25" customWidth="1"/>
-    <col min="10" max="10" width="23.375" customWidth="1"/>
+    <col min="10" max="10" width="19.875" customWidth="1"/>
     <col min="11" max="12" width="16.25" customWidth="1"/>
     <col min="13" max="13" width="16.25" style="2" customWidth="1"/>
     <col min="14" max="19" width="42.375" customWidth="1"/>
     <col min="20" max="20" width="16.25" customWidth="1"/>
     <col min="21" max="21" width="42.375" customWidth="1"/>
     <col min="22" max="22" width="16.25" customWidth="1"/>
-    <col min="23" max="24" width="42.375" customWidth="1"/>
+    <col min="23" max="23" width="42.375" customWidth="1"/>
+    <col min="24" max="24" width="23" customWidth="1"/>
     <col min="25" max="25" width="14.75" customWidth="1"/>
     <col min="26" max="26" width="13" customWidth="1"/>
     <col min="27" max="27" width="16.25" customWidth="1"/>
@@ -629,14 +635,16 @@
     <col min="30" max="30" width="42.375" style="1" customWidth="1"/>
     <col min="31" max="32" width="16.25" customWidth="1"/>
     <col min="33" max="34" width="16.25" style="1" customWidth="1"/>
-    <col min="35" max="42" width="16.25" customWidth="1"/>
+    <col min="35" max="39" width="16.25" customWidth="1"/>
+    <col min="40" max="40" width="16.25" style="9" customWidth="1"/>
+    <col min="41" max="42" width="16.25" customWidth="1"/>
     <col min="43" max="44" width="19.5" customWidth="1"/>
     <col min="45" max="46" width="16.25" customWidth="1"/>
     <col min="47" max="47" width="16.625" customWidth="1"/>
     <col min="48" max="48" width="17.875" customWidth="1"/>
     <col min="49" max="55" width="16.25" customWidth="1"/>
     <col min="56" max="56" width="21.875" customWidth="1"/>
-    <col min="57" max="57" width="17.875" customWidth="1"/>
+    <col min="57" max="57" width="17.875" style="9" customWidth="1"/>
     <col min="58" max="59" width="16.25" customWidth="1"/>
     <col min="60" max="60" width="9.875" customWidth="1"/>
     <col min="61" max="61" width="23" customWidth="1"/>
@@ -890,7 +898,7 @@
       <c r="AM11" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="AN11" s="8" t="s">
+      <c r="AN11" s="10" t="s">
         <v>54</v>
       </c>
       <c r="AO11" s="5" t="s">
@@ -941,7 +949,7 @@
       <c r="BD11" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="BE11" s="5" t="s">
+      <c r="BE11" s="10" t="s">
         <v>56</v>
       </c>
       <c r="BF11" s="5" t="s">

</xml_diff>